<commit_message>
Traspasos: ignorar pedidos a domicilio al importar recolecciones
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CFp4T5cDi1AkfpkBAFCtiY
</commit_message>
<xml_diff>
--- a/traspasos/Traspasos_FADERMEX_BD.xlsx
+++ b/traspasos/Traspasos_FADERMEX_BD.xlsx
@@ -27,9 +27,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RES_Sesiones" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RES_Avisos" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IMP_Recolecciones" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IMP_NoRegistrados" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REP_Resumen" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SYS_Folios" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="REP_Resumen" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SYS_Folios" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'RES_Traspasos'!$A$2:$Y$2</definedName>
@@ -848,7 +847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D93"/>
+  <dimension ref="A1:D92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1482,92 +1481,87 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="9" t="inlineStr">
-        <is>
-          <t>IMP_NoRegistrados</t>
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>REP_Resumen</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>IMP</t>
+          <t>REP</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Folios escaneados por gestores que no existen en este sistema.</t>
+          <t>Conteos por estatus y por área.</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Nadie (se copia solo)</t>
+          <t>Nadie (fórmulas)</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="7" t="inlineStr">
-        <is>
-          <t>REP_Resumen</t>
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t>SYS_Folios</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>REP</t>
+          <t>SYS</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Conteos por estatus y por área.</t>
+          <t>Contadores de folios.</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Nadie (fórmulas)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
-        <is>
-          <t>SYS_Folios</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>SYS</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Contadores de folios.</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
           <t>Solo la app</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>DICCIONARIO DE COLUMNAS</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>DICCIONARIO DE COLUMNAS</t>
+          <t>HOJA</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>COLUMNA</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>QUÉ SIGNIFICA</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="inlineStr">
-        <is>
-          <t>HOJA</t>
-        </is>
-      </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>COLUMNA</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>QUÉ SIGNIFICA</t>
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>CAT_Estatus</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Clave</t>
+        </is>
+      </c>
+      <c r="C46" s="10" t="inlineStr">
+        <is>
+          <t>Código interno. NO cambiar.</t>
         </is>
       </c>
     </row>
@@ -1579,12 +1573,12 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Clave</t>
+          <t>Nombre en pantalla</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>Código interno. NO cambiar.</t>
+          <t>Texto que ve el usuario.</t>
         </is>
       </c>
     </row>
@@ -1596,12 +1590,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Nombre en pantalla</t>
+          <t>Color texto (hex)</t>
         </is>
       </c>
       <c r="C48" s="10" t="inlineStr">
         <is>
-          <t>Texto que ve el usuario.</t>
+          <t>Color del texto/punto del estatus en la app.</t>
         </is>
       </c>
     </row>
@@ -1613,12 +1607,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Color texto (hex)</t>
+          <t>Color fondo (hex)</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>Color del texto/punto del estatus en la app.</t>
+          <t>Color de fondo de la etiqueta de estatus en la app.</t>
         </is>
       </c>
     </row>
@@ -1630,29 +1624,29 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Color fondo (hex)</t>
+          <t>Estado en app de gestores</t>
         </is>
       </c>
       <c r="C50" s="10" t="inlineStr">
         <is>
-          <t>Color de fondo de la etiqueta de estatus en la app.</t>
+          <t>Qué Estado de APP_Traspasos (archivo de Operaciones) produce este estatus.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAT_Estatus</t>
+          <t>CAT_Sucursales</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Estado en app de gestores</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
         <is>
-          <t>Qué Estado de APP_Traspasos (archivo de Operaciones) produce este estatus.</t>
+          <t>Código corto del lugar.</t>
         </is>
       </c>
     </row>
@@ -1664,12 +1658,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>Código corto del lugar.</t>
+          <t>Oficinas / Sucursal / Foránea / Área independiente</t>
         </is>
       </c>
     </row>
@@ -1681,12 +1675,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Tipo</t>
+          <t>Cómo se envía</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
         <is>
-          <t>Oficinas / Sucursal / Foránea / Área independiente</t>
+          <t>Gestoría, paquetería o entrega interna.</t>
         </is>
       </c>
     </row>
@@ -1698,29 +1692,29 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Cómo se envía</t>
+          <t>Activa</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
         <is>
-          <t>Gestoría, paquetería o entrega interna.</t>
+          <t>SI / NO</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CAT_Sucursales</t>
+          <t>CAT_Areas</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Prefijo de folio</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
         <is>
-          <t>SI / NO</t>
+          <t>Único. 2 a 5 letras (o XX-RB). No cambiar una vez usado.</t>
         </is>
       </c>
     </row>
@@ -1732,12 +1726,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Prefijo de folio</t>
+          <t>Sucursal (ID)</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
         <is>
-          <t>Único. 2 a 5 letras (o XX-RB). No cambiar una vez usado.</t>
+          <t>ID de CAT_Sucursales</t>
         </is>
       </c>
     </row>
@@ -1749,12 +1743,12 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Sucursal (ID)</t>
+          <t>Correo de la cuenta</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
         <is>
-          <t>ID de CAT_Sucursales</t>
+          <t>Correo con el que entra. En sucursales PV y Rebotica comparten la cuenta.</t>
         </is>
       </c>
     </row>
@@ -1766,29 +1760,29 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Correo de la cuenta</t>
+          <t>Activa</t>
         </is>
       </c>
       <c r="C58" s="10" t="inlineStr">
         <is>
-          <t>Correo con el que entra. En sucursales PV y Rebotica comparten la cuenta.</t>
+          <t>SI / NO. Para quitar un área pon NO; no borres la fila.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CAT_Areas</t>
+          <t>CAT_Equipos</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>ID equipo</t>
         </is>
       </c>
       <c r="C59" s="10" t="inlineStr">
         <is>
-          <t>SI / NO. Para quitar un área pon NO; no borres la fila.</t>
+          <t>Se configura una sola vez en la computadora (lo hace un administrador).</t>
         </is>
       </c>
     </row>
@@ -1800,12 +1794,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>ID equipo</t>
+          <t>Área (prefijo)</t>
         </is>
       </c>
       <c r="C60" s="10" t="inlineStr">
         <is>
-          <t>Se configura una sola vez en la computadora (lo hace un administrador).</t>
+          <t>Área con la que crea y da salida a traspasos.</t>
         </is>
       </c>
     </row>
@@ -1817,29 +1811,29 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Área (prefijo)</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="C61" s="10" t="inlineStr">
         <is>
-          <t>Área con la que crea y da salida a traspasos.</t>
+          <t>SI / NO</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAT_Equipos</t>
+          <t>CAT_Personas</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Código de credencial</t>
         </is>
       </c>
       <c r="C62" s="10" t="inlineStr">
         <is>
-          <t>SI / NO</t>
+          <t>Lo que lee la pistola al escanear la credencial.</t>
         </is>
       </c>
     </row>
@@ -1851,12 +1845,12 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Código de credencial</t>
+          <t>Área (prefijo)</t>
         </is>
       </c>
       <c r="C63" s="10" t="inlineStr">
         <is>
-          <t>Lo que lee la pistola al escanear la credencial.</t>
+          <t>Área donde trabaja.</t>
         </is>
       </c>
     </row>
@@ -1868,12 +1862,12 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Área (prefijo)</t>
+          <t>Tiene credencial</t>
         </is>
       </c>
       <c r="C64" s="10" t="inlineStr">
         <is>
-          <t>Área donde trabaja.</t>
+          <t>SI / NO</t>
         </is>
       </c>
     </row>
@@ -1885,12 +1879,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Tiene credencial</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="C65" s="10" t="inlineStr">
         <is>
-          <t>SI / NO</t>
+          <t>SI / NO. Si pierde la credencial: Activo = NO y se le da una nueva.</t>
         </is>
       </c>
     </row>
@@ -1902,46 +1896,46 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Alta</t>
         </is>
       </c>
       <c r="C66" s="10" t="inlineStr">
         <is>
-          <t>SI / NO. Si pierde la credencial: Activo = NO y se le da una nueva.</t>
+          <t>Fecha de registro</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CAT_Personas</t>
+          <t>CAT_Gestores</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="C67" s="10" t="inlineStr">
         <is>
-          <t>Fecha de registro</t>
+          <t>SI / NO</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CAT_Gestores</t>
+          <t>CAT_Administradores</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Rol</t>
         </is>
       </c>
       <c r="C68" s="10" t="inlineStr">
         <is>
-          <t>SI / NO</t>
+          <t>Dueño / Administrador</t>
         </is>
       </c>
     </row>
@@ -1953,24 +1947,24 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Rol</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="C69" s="10" t="inlineStr">
         <is>
-          <t>Dueño / Administrador</t>
+          <t>SI / NO</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CAT_Administradores</t>
+          <t>CAT_Paqueterias</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Activa</t>
         </is>
       </c>
       <c r="C70" s="10" t="inlineStr">
@@ -1982,17 +1976,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CAT_Paqueterias</t>
+          <t>CAT_Motivos</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Activa</t>
+          <t>Tipo</t>
         </is>
       </c>
       <c r="C71" s="10" t="inlineStr">
         <is>
-          <t>SI / NO</t>
+          <t>REIMPRESION / ELIMINACION / INCIDENCIA</t>
         </is>
       </c>
     </row>
@@ -2004,46 +1998,46 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Tipo</t>
+          <t>Activo</t>
         </is>
       </c>
       <c r="C72" s="10" t="inlineStr">
         <is>
-          <t>REIMPRESION / ELIMINACION / INCIDENCIA</t>
+          <t>SI / NO</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CAT_Motivos</t>
+          <t>CFG_Ajustes</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Activo</t>
+          <t>Parámetro</t>
         </is>
       </c>
       <c r="C73" s="10" t="inlineStr">
         <is>
-          <t>SI / NO</t>
+          <t>NO cambiar el nombre.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CFG_Ajustes</t>
+          <t>RES_Traspasos</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Parámetro</t>
+          <t>Folio</t>
         </is>
       </c>
       <c r="C74" s="10" t="inlineStr">
         <is>
-          <t>NO cambiar el nombre.</t>
+          <t>Prefijo + consecutivo. Único.</t>
         </is>
       </c>
     </row>
@@ -2055,12 +2049,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Folio</t>
+          <t>Sin credencial</t>
         </is>
       </c>
       <c r="C75" s="10" t="inlineStr">
         <is>
-          <t>Prefijo + consecutivo. Único.</t>
+          <t>SI si se creó sin credencial.</t>
         </is>
       </c>
     </row>
@@ -2072,12 +2066,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Sin credencial</t>
+          <t>Estatus</t>
         </is>
       </c>
       <c r="C76" s="10" t="inlineStr">
         <is>
-          <t>SI si se creó sin credencial.</t>
+          <t>Clave de CAT_Estatus. El color de la fila sale de ahí.</t>
         </is>
       </c>
     </row>
@@ -2089,12 +2083,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Estatus</t>
+          <t>Ubicación actual</t>
         </is>
       </c>
       <c r="C77" s="10" t="inlineStr">
         <is>
-          <t>Clave de CAT_Estatus. El color de la fila sale de ahí.</t>
+          <t>Llena solo si el estatus es UBICADO.</t>
         </is>
       </c>
     </row>
@@ -2106,12 +2100,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Ubicación actual</t>
+          <t>Ruta</t>
         </is>
       </c>
       <c r="C78" s="10" t="inlineStr">
         <is>
-          <t>Llena solo si el estatus es UBICADO.</t>
+          <t>DIRECTA o VIA_LOGISTICA (Morelia).</t>
         </is>
       </c>
     </row>
@@ -2123,12 +2117,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Ruta</t>
+          <t>Reimpresiones</t>
         </is>
       </c>
       <c r="C79" s="10" t="inlineStr">
         <is>
-          <t>DIRECTA o VIA_LOGISTICA (Morelia).</t>
+          <t>Cuántas veces se reimprimieron etiquetas.</t>
         </is>
       </c>
     </row>
@@ -2140,29 +2134,29 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Reimpresiones</t>
+          <t>Eliminación solicitada</t>
         </is>
       </c>
       <c r="C80" s="10" t="inlineStr">
         <is>
-          <t>Cuántas veces se reimprimieron etiquetas.</t>
+          <t>SI / NO</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>RES_Traspasos</t>
+          <t>RES_Movimientos</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Eliminación solicitada</t>
+          <t>Acción</t>
         </is>
       </c>
       <c r="C81" s="10" t="inlineStr">
         <is>
-          <t>SI / NO</t>
+          <t>CREADO, ETIQUETAS, RECOLECTADO, RECIBIDO, PAQUETERIA, REIMPRESION, SOLICITUD, EDICION_ADMIN…</t>
         </is>
       </c>
     </row>
@@ -2174,12 +2168,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Acción</t>
+          <t>Medio</t>
         </is>
       </c>
       <c r="C82" s="10" t="inlineStr">
         <is>
-          <t>CREADO, ETIQUETAS, RECOLECTADO, RECIBIDO, PAQUETERIA, REIMPRESION, SOLICITUD, EDICION_ADMIN…</t>
+          <t>PISTOLA, CELULAR, TECLADO, CREDENCIAL_GESTOR</t>
         </is>
       </c>
     </row>
@@ -2191,29 +2185,29 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Medio</t>
+          <t>Equipo</t>
         </is>
       </c>
       <c r="C83" s="10" t="inlineStr">
         <is>
-          <t>PISTOLA, CELULAR, TECLADO, CREDENCIAL_GESTOR</t>
+          <t>ID de CAT_Equipos</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>RES_Movimientos</t>
+          <t>RES_Escaneos</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Equipo</t>
+          <t>Modo</t>
         </is>
       </c>
       <c r="C84" s="10" t="inlineStr">
         <is>
-          <t>ID de CAT_Equipos</t>
+          <t>RECIBIR, ENTREGAR_A_GESTOR, RECOLECTAR</t>
         </is>
       </c>
     </row>
@@ -2225,29 +2219,29 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Modo</t>
+          <t>Resultado</t>
         </is>
       </c>
       <c r="C85" s="10" t="inlineStr">
         <is>
-          <t>RECIBIR, ENTREGAR_A_GESTOR, RECOLECTAR</t>
+          <t>OK, AVISO, ERROR</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>RES_Escaneos</t>
+          <t>RES_Etiquetas</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Resultado</t>
+          <t>Bulto</t>
         </is>
       </c>
       <c r="C86" s="10" t="inlineStr">
         <is>
-          <t>OK, AVISO, ERROR</t>
+          <t>Ej. 2/3</t>
         </is>
       </c>
     </row>
@@ -2259,112 +2253,95 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Bulto</t>
+          <t>Impresión</t>
         </is>
       </c>
       <c r="C87" s="10" t="inlineStr">
         <is>
-          <t>Ej. 2/3</t>
+          <t>ORIGINAL o R1, R2…</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>RES_Etiquetas</t>
+          <t>RES_Solicitudes</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Impresión</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="C88" s="10" t="inlineStr">
         <is>
-          <t>ORIGINAL o R1, R2…</t>
+          <t>PENDIENTE, APROBADA, RECHAZADA</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>RES_Solicitudes</t>
+          <t>RES_Administracion</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Estado</t>
+          <t>Objeto</t>
         </is>
       </c>
       <c r="C89" s="10" t="inlineStr">
         <is>
-          <t>PENDIENTE, APROBADA, RECHAZADA</t>
+          <t>Folio, área, persona…</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>RES_Administracion</t>
+          <t>RES_Sesiones</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Objeto</t>
+          <t>Evento</t>
         </is>
       </c>
       <c r="C90" s="10" t="inlineStr">
         <is>
-          <t>Folio, área, persona…</t>
+          <t>ENTRADA, SALIDA, EXPIRÓ</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>RES_Sesiones</t>
+          <t>RES_Avisos</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Evento</t>
+          <t>Visto</t>
         </is>
       </c>
       <c r="C91" s="10" t="inlineStr">
         <is>
-          <t>ENTRADA, SALIDA, EXPIRÓ</t>
+          <t>SI / NO</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>RES_Avisos</t>
+          <t>IMP_Recolecciones</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Visto</t>
+          <t>Estado</t>
         </is>
       </c>
       <c r="C92" s="10" t="inlineStr">
-        <is>
-          <t>SI / NO</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>IMP_Recolecciones</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-      <c r="C93" s="10" t="inlineStr">
         <is>
           <t>POR ENTREGAR / ENTREGADO / NO ENTREGADO</t>
         </is>
@@ -2393,7 +2370,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A40" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A41" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A42" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A43" r:id="rId22"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4171,7 +4147,7 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>IMP_Recolecciones  —  IMPORTADO · Se copia solo desde tu archivo de Operaciones · NO editar.  Copia en vivo de la hoja APP_Traspasos de tu archivo de Operaciones (lo que escanean los gestores). La app la cruza por Folio y actualiza RES_Traspasos.</t>
+          <t>IMP_Recolecciones  —  IMPORTADO · Se copia solo desde tu archivo de Operaciones · NO editar.  Copia en vivo de APP_Traspasos (archivo de Operaciones). Ahí también hay pedidos a domicilio: la app SOLO toma los folios que existen en RES_Traspasos e ignora el resto.</t>
         </is>
       </c>
     </row>
@@ -4242,65 +4218,6 @@
 </file>
 
 <file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="000B6C80"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="36" customHeight="1">
-      <c r="A1" s="39" t="inlineStr">
-        <is>
-          <t>IMP_NoRegistrados  —  IMPORTADO · Se copia solo desde tu archivo de Operaciones · NO editar.  Folios que escaneó un gestor pero NO existen en este sistema (mal escaneados, o traspasos hechos fuera del sistema). Revisar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1">
-      <c r="A2" s="40" t="inlineStr">
-        <is>
-          <t>Folio</t>
-        </is>
-      </c>
-      <c r="B2" s="40" t="inlineStr">
-        <is>
-          <t>FechaRecoleccion</t>
-        </is>
-      </c>
-      <c r="C2" s="40" t="inlineStr">
-        <is>
-          <t>Gestor</t>
-        </is>
-      </c>
-      <c r="D2" s="40" t="inlineStr">
-        <is>
-          <t>Estado</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3">
-        <f>IFERROR(FILTER({IMP_Recolecciones!A3:C,IMP_Recolecciones!I3:I},IMP_Recolecciones!A3:A&lt;&gt;"",ISNA(MATCH(IMP_Recolecciones!A3:A,RES_Traspasos!A3:A,0))),"Sin folios desconocidos")</f>
-        <v/>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00C4440B"/>
@@ -4889,7 +4806,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="005A6977"/>

</xml_diff>

<commit_message>
Traspasos: etiqueta general de 50 × 20 mm para todas las sucursales; recibir en tu computadora sin credencial
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CFp4T5cDi1AkfpkBAFCtiY
</commit_message>
<xml_diff>
--- a/traspasos/Traspasos_FADERMEX_BD.xlsx
+++ b/traspasos/Traspasos_FADERMEX_BD.xlsx
@@ -2760,11 +2760,11 @@
         </is>
       </c>
       <c r="B10" s="36" t="n">
-        <v>62</v>
+        <v>50</v>
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>Ancho de la etiqueta. PENDIENTE confirmar con el modelo de la etiquetadora.</t>
+          <t>Ancho de la etiqueta en mm (rollo de todas las sucursales: 5 cm).</t>
         </is>
       </c>
     </row>
@@ -2775,11 +2775,11 @@
         </is>
       </c>
       <c r="B11" s="36" t="n">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>Alto de la etiqueta. PENDIENTE confirmar.</t>
+          <t>Alto de la etiqueta en mm (rollo de todas las sucursales: 2 cm).</t>
         </is>
       </c>
     </row>
@@ -2791,12 +2791,12 @@
       </c>
       <c r="B12" s="36" t="inlineStr">
         <is>
-          <t>PENDIENTE</t>
+          <t>Argox OS-2140 (y otras)</t>
         </is>
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>Modelo de las etiquetadoras Brother.</t>
+          <t>Modelo de las etiquetadoras. El tamaño de cada área se puede cambiar en CAT_Impresoras.</t>
         </is>
       </c>
     </row>

</xml_diff>